<commit_message>
arquivo data base completo
</commit_message>
<xml_diff>
--- a/data/03-03-2026 20_19_16.xlsx
+++ b/data/03-03-2026 20_19_16.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://projexacombr-my.sharepoint.com/personal/pedro_figueira_projexa-energy_com_br/Documents/Área de Trabalho/Estudos_python/1.Dashboard_gastos_projetos/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://projexacombr-my.sharepoint.com/personal/pedro_figueira_projexa-energy_com_br/Documents/Área de Trabalho/Estudos_python/1.Dashboard_reembolso_projetos/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="11_F5A09674C57BD973335A6C52E77BD2723AC5E138" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EA207F49-08B5-4528-B6B6-581A1A778516}"/>
+  <xr:revisionPtr revIDLastSave="16" documentId="11_F5A09674C57BD973335A6C52E77BD2723AC5E138" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6B829BC6-4710-41D2-B518-025CEB528431}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2853,6 +2853,7 @@
     <col min="3" max="3" width="11.81640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.7265625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="19.90625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.90625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="79" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="46.54296875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="234" bestFit="1" customWidth="1"/>

</xml_diff>